<commit_message>
score b validation finished
</commit_message>
<xml_diff>
--- a/2025_demo/GlycoMSP_scoring_update_example_v5.xlsx
+++ b/2025_demo/GlycoMSP_scoring_update_example_v5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\其他電腦\My Computer\GlycoMSParser\2025_demo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3D14814-DF3D-4E22-89B4-986A5CE43918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C46A41DD-3F70-4CFE-8B1D-4AA0069F8D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{CFD31651-57D7-40EF-BE95-C7417EC3B9A0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="5" activeTab="7" xr2:uid="{CFD31651-57D7-40EF-BE95-C7417EC3B9A0}"/>
   </bookViews>
   <sheets>
     <sheet name="MSlist" sheetId="6" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="981" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="989" uniqueCount="298">
   <si>
     <t>note</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1299,9 +1299,6 @@
     <t>when_value</t>
   </si>
   <si>
-    <t>S0_penalize_sialyl</t>
-  </si>
-  <si>
     <t>S</t>
   </si>
   <si>
@@ -1807,6 +1804,32 @@
   </si>
   <si>
     <t>(keep empty for now (as unit test of empty column)) UPDATE: name_unsolved as rule</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>include_descendants</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SialylGcGalNAc</t>
+  </si>
+  <si>
+    <t>SialylAcGalNAc</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SialylGcHex</t>
+  </si>
+  <si>
+    <t>SialylAcHex</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>S0_penalize_sialylAc</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>activation_mode</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3068,26 +3091,26 @@
   <sheetData>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
+        <v>175</v>
+      </c>
+      <c r="B6" t="s">
         <v>176</v>
-      </c>
-      <c r="B6" t="s">
-        <v>177</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E6" t="s">
         <v>0</v>
@@ -3098,37 +3121,37 @@
         <v>56</v>
       </c>
       <c r="C7" t="s">
+        <v>178</v>
+      </c>
+      <c r="D7" t="s">
+        <v>173</v>
+      </c>
+      <c r="E7" t="s">
         <v>179</v>
-      </c>
-      <c r="D7" t="s">
-        <v>174</v>
-      </c>
-      <c r="E7" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B17" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C17" t="s">
         <v>0</v>
       </c>
       <c r="D17" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -3136,26 +3159,26 @@
         <v>149</v>
       </c>
       <c r="C18" t="s">
+        <v>185</v>
+      </c>
+      <c r="D18" t="s">
         <v>186</v>
-      </c>
-      <c r="D18" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="B19" t="s">
+        <v>183</v>
+      </c>
+      <c r="C19" t="s">
+        <v>187</v>
+      </c>
+      <c r="D19" t="s">
         <v>184</v>
-      </c>
-      <c r="C19" t="s">
-        <v>188</v>
-      </c>
-      <c r="D19" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="198">
       <c r="A25" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -3181,22 +3204,22 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
+        <v>278</v>
+      </c>
+      <c r="B1" t="s">
+        <v>277</v>
+      </c>
+      <c r="C1" t="s">
+        <v>281</v>
+      </c>
+      <c r="D1" t="s">
+        <v>282</v>
+      </c>
+      <c r="E1" t="s">
         <v>279</v>
       </c>
-      <c r="B1" t="s">
-        <v>278</v>
-      </c>
-      <c r="C1" t="s">
-        <v>282</v>
-      </c>
-      <c r="D1" t="s">
-        <v>283</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>280</v>
-      </c>
-      <c r="F1" t="s">
-        <v>281</v>
       </c>
       <c r="G1" t="s">
         <v>7</v>
@@ -3270,7 +3293,7 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B5" t="s">
         <v>95</v>
@@ -3288,7 +3311,7 @@
         <v>30</v>
       </c>
       <c r="G5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -3402,7 +3425,7 @@
         <v>656.34879999999998</v>
       </c>
       <c r="D11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E11" t="s">
         <v>29</v>
@@ -3431,7 +3454,7 @@
         <v>30</v>
       </c>
       <c r="G12" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -3468,7 +3491,7 @@
         <v>402.21230000000003</v>
       </c>
       <c r="D14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E14" t="s">
         <v>29</v>
@@ -3517,7 +3540,7 @@
         <v>656.34879999999998</v>
       </c>
       <c r="D16" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
@@ -3526,7 +3549,7 @@
         <v>30</v>
       </c>
       <c r="G16" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -3540,7 +3563,7 @@
         <v>432.22280000000001</v>
       </c>
       <c r="D17" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E17" t="s">
         <v>29</v>
@@ -3651,7 +3674,7 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B23" t="s">
         <v>21</v>
@@ -3671,7 +3694,7 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B24" t="s">
         <v>35</v>
@@ -3680,7 +3703,7 @@
         <v>566.28070000000002</v>
       </c>
       <c r="D24" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E24" t="s">
         <v>29</v>
@@ -3694,7 +3717,7 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B25" t="s">
         <v>41</v>
@@ -3703,7 +3726,7 @@
         <v>825.42269999999996</v>
       </c>
       <c r="D25" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E25" t="s">
         <v>29</v>
@@ -3757,7 +3780,7 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B28" t="s">
         <v>15</v>
@@ -3766,7 +3789,7 @@
         <v>999.51189999999997</v>
       </c>
       <c r="D28" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E28" t="s">
         <v>29</v>
@@ -3777,7 +3800,7 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B29" t="s">
         <v>15</v>
@@ -3786,7 +3809,7 @@
         <v>855.43330000000003</v>
       </c>
       <c r="D29" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E29" t="s">
         <v>29</v>
@@ -3797,16 +3820,16 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" t="s">
+        <v>205</v>
+      </c>
+      <c r="B30" t="s">
         <v>206</v>
-      </c>
-      <c r="B30" t="s">
-        <v>207</v>
       </c>
       <c r="C30">
         <v>624.32259999999997</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E30" t="s">
         <v>29</v>
@@ -3817,7 +3840,7 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B31" t="s">
         <v>15</v>
@@ -3826,7 +3849,7 @@
         <v>1029.5225</v>
       </c>
       <c r="D31" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E31" t="s">
         <v>29</v>
@@ -3837,7 +3860,7 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B32" t="s">
         <v>15</v>
@@ -3846,7 +3869,7 @@
         <v>1029.5225</v>
       </c>
       <c r="D32" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E32" t="s">
         <v>29</v>
@@ -3857,7 +3880,7 @@
     </row>
     <row r="33" spans="1:7">
       <c r="A33" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B33" t="s">
         <v>15</v>
@@ -3866,7 +3889,7 @@
         <v>1203.6116999999999</v>
       </c>
       <c r="D33" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E33" t="s">
         <v>29</v>
@@ -3875,12 +3898,12 @@
         <v>30</v>
       </c>
       <c r="G33" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="34" spans="1:7">
       <c r="A34" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B34" t="s">
         <v>15</v>
@@ -3889,7 +3912,7 @@
         <v>1233.6222</v>
       </c>
       <c r="D34" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E34" t="s">
         <v>29</v>
@@ -3900,10 +3923,10 @@
     </row>
     <row r="35" spans="1:7">
       <c r="A35" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B35" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C35">
         <v>866.44920000000002</v>
@@ -3920,16 +3943,16 @@
     </row>
     <row r="36" spans="1:7">
       <c r="A36" t="s">
+        <v>248</v>
+      </c>
+      <c r="B36" t="s">
         <v>249</v>
-      </c>
-      <c r="B36" t="s">
-        <v>250</v>
       </c>
       <c r="C36">
         <v>896.45979999999997</v>
       </c>
       <c r="D36" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E36" t="s">
         <v>29</v>
@@ -3940,16 +3963,16 @@
     </row>
     <row r="37" spans="1:7">
       <c r="A37" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B37" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C37">
         <v>621.3229</v>
       </c>
       <c r="D37" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E37" t="s">
         <v>29</v>
@@ -3960,16 +3983,16 @@
     </row>
     <row r="38" spans="1:7">
       <c r="A38" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B38" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C38">
         <v>651.33349999999996</v>
       </c>
       <c r="D38" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E38" t="s">
         <v>29</v>
@@ -3980,7 +4003,7 @@
     </row>
     <row r="39" spans="1:7">
       <c r="A39" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B39" t="s">
         <v>15</v>
@@ -3989,7 +4012,7 @@
         <v>610.30690000000004</v>
       </c>
       <c r="D39" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E39" t="s">
         <v>29</v>
@@ -4000,7 +4023,7 @@
     </row>
     <row r="40" spans="1:7">
       <c r="A40" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B40" t="s">
         <v>35</v>
@@ -4009,7 +4032,7 @@
         <v>596.29129999999998</v>
       </c>
       <c r="D40" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E40" t="s">
         <v>29</v>
@@ -4053,7 +4076,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="33">
       <c r="A1" s="4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>156</v>
@@ -4062,7 +4085,7 @@
         <v>57</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>111</v>
@@ -4071,7 +4094,7 @@
         <v>109</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>58</v>
@@ -4106,7 +4129,7 @@
         <v>124</v>
       </c>
       <c r="D2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F2" t="s">
         <v>81</v>
@@ -4144,7 +4167,7 @@
         <v>124</v>
       </c>
       <c r="D3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E3" t="s">
         <v>80</v>
@@ -4185,7 +4208,7 @@
         <v>124</v>
       </c>
       <c r="D4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F4" t="s">
         <v>86</v>
@@ -4217,13 +4240,13 @@
         <v>84</v>
       </c>
       <c r="B5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>124</v>
       </c>
       <c r="D5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E5" t="s">
         <v>84</v>
@@ -4302,7 +4325,7 @@
         <v>106</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>79</v>
@@ -4346,7 +4369,7 @@
         <v>124</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>110</v>
@@ -4384,7 +4407,7 @@
         <v>65</v>
       </c>
       <c r="D9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F9" t="s">
         <v>45</v>
@@ -4422,7 +4445,7 @@
         <v>65</v>
       </c>
       <c r="D10" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>72</v>
@@ -4466,7 +4489,7 @@
         <v>65</v>
       </c>
       <c r="D11" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F11" t="s">
         <v>54</v>
@@ -4504,7 +4527,7 @@
         <v>124</v>
       </c>
       <c r="D12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E12" t="s">
         <v>46</v>
@@ -4536,25 +4559,25 @@
     </row>
     <row r="13" spans="1:14" ht="33">
       <c r="A13" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>65</v>
       </c>
       <c r="D13" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>74</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H13" s="7" t="s">
         <v>67</v>
@@ -4575,30 +4598,30 @@
         <v>69</v>
       </c>
       <c r="N13" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="33">
       <c r="A14" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>65</v>
       </c>
       <c r="D14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E14" s="7" t="s">
         <v>47</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G14" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H14" s="7" t="s">
         <v>67</v>
@@ -4619,27 +4642,27 @@
         <v>69</v>
       </c>
       <c r="N14" s="7" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="15" spans="1:14">
       <c r="A15" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B15" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>65</v>
       </c>
       <c r="D15" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F15" t="s">
         <v>28</v>
       </c>
       <c r="G15" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H15" s="7" t="s">
         <v>67</v>
@@ -4671,13 +4694,13 @@
         <v>65</v>
       </c>
       <c r="D16" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>19</v>
       </c>
       <c r="F16" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G16" t="s">
         <v>92</v>
@@ -4715,7 +4738,7 @@
         <v>65</v>
       </c>
       <c r="D17" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F17" t="s">
         <v>48</v>
@@ -4747,13 +4770,13 @@
         <v>94</v>
       </c>
       <c r="B18" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>65</v>
       </c>
       <c r="D18" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E18" t="s">
         <v>47</v>
@@ -4794,7 +4817,7 @@
         <v>106</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>32</v>
@@ -4835,7 +4858,7 @@
         <v>106</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F20" t="s">
         <v>42</v>
@@ -4873,7 +4896,7 @@
         <v>106</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>33</v>
@@ -4914,7 +4937,7 @@
         <v>106</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F22" t="s">
         <v>43</v>
@@ -4946,25 +4969,25 @@
     </row>
     <row r="23" spans="1:14">
       <c r="A23" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B23" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>124</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E23" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F23" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="G23" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="H23" s="7" t="s">
         <v>67</v>
@@ -4987,25 +5010,25 @@
     </row>
     <row r="24" spans="1:14">
       <c r="A24" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B24" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>124</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E24" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F24" t="s">
         <v>34</v>
       </c>
       <c r="G24" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="H24" s="7" t="s">
         <v>67</v>
@@ -5028,10 +5051,10 @@
     </row>
     <row r="25" spans="1:14">
       <c r="A25" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B25" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>65</v>
@@ -5041,10 +5064,10 @@
       </c>
       <c r="E25" s="7"/>
       <c r="F25" s="7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G25" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H25" s="7" t="s">
         <v>67</v>
@@ -5070,22 +5093,22 @@
     </row>
     <row r="26" spans="1:14">
       <c r="A26" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B26" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>124</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F26" t="s">
         <v>146</v>
       </c>
       <c r="G26" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="H26" s="7" t="s">
         <v>67</v>
@@ -5108,25 +5131,25 @@
     </row>
     <row r="27" spans="1:14">
       <c r="A27" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B27" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>124</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E27" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F27" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G27" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H27" s="7" t="s">
         <v>67</v>
@@ -5149,10 +5172,10 @@
     </row>
     <row r="28" spans="1:14">
       <c r="A28" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B28" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>65</v>
@@ -5162,10 +5185,10 @@
       </c>
       <c r="E28" s="7"/>
       <c r="F28" s="7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G28" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H28" s="7" t="s">
         <v>67</v>
@@ -5191,25 +5214,25 @@
     </row>
     <row r="29" spans="1:14">
       <c r="A29" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B29" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>124</v>
       </c>
       <c r="D29" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="E29" t="s">
+        <v>198</v>
+      </c>
+      <c r="F29" t="s">
+        <v>260</v>
+      </c>
+      <c r="G29" t="s">
         <v>258</v>
-      </c>
-      <c r="E29" t="s">
-        <v>199</v>
-      </c>
-      <c r="F29" t="s">
-        <v>261</v>
-      </c>
-      <c r="G29" t="s">
-        <v>259</v>
       </c>
       <c r="H29" s="7" t="s">
         <v>67</v>
@@ -5232,22 +5255,22 @@
     </row>
     <row r="30" spans="1:14">
       <c r="A30" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B30" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C30" s="7" t="s">
         <v>124</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F30" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G30" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H30" s="7" t="s">
         <v>67</v>
@@ -5270,22 +5293,22 @@
     </row>
     <row r="31" spans="1:14">
       <c r="A31" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B31" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>65</v>
       </c>
       <c r="D31" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F31" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G31" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H31" s="7" t="s">
         <v>67</v>
@@ -5317,7 +5340,7 @@
         <v>65</v>
       </c>
       <c r="D32" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E32" s="7"/>
       <c r="F32" s="7" t="s">
@@ -5350,7 +5373,7 @@
     </row>
     <row r="33" spans="1:13">
       <c r="A33" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B33" t="s">
         <v>96</v>
@@ -5359,7 +5382,7 @@
         <v>124</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E33" t="s">
         <v>36</v>
@@ -5394,7 +5417,7 @@
         <v>103</v>
       </c>
       <c r="B34" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>124</v>
@@ -5406,7 +5429,7 @@
         <v>104</v>
       </c>
       <c r="G34" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="H34" s="7" t="s">
         <v>67</v>
@@ -5432,7 +5455,7 @@
         <v>102</v>
       </c>
       <c r="B35" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C35" s="7" t="s">
         <v>124</v>
@@ -5444,7 +5467,7 @@
         <v>77</v>
       </c>
       <c r="G35" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H35" s="7" t="s">
         <v>67</v>
@@ -5467,22 +5490,22 @@
     </row>
     <row r="36" spans="1:13">
       <c r="A36" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B36" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C36" s="7" t="s">
         <v>124</v>
       </c>
       <c r="D36" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F36" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G36" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H36" s="7" t="s">
         <v>67</v>
@@ -5527,19 +5550,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
+        <v>229</v>
+      </c>
+      <c r="B1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C1" t="s">
         <v>230</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>234</v>
       </c>
-      <c r="C1" t="s">
-        <v>231</v>
-      </c>
-      <c r="D1" t="s">
-        <v>235</v>
-      </c>
       <c r="E1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -5550,13 +5573,13 @@
         <v>999</v>
       </c>
       <c r="C2" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D2">
         <v>624</v>
       </c>
       <c r="E2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -5567,13 +5590,13 @@
         <v>999</v>
       </c>
       <c r="C3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D3">
         <v>793</v>
       </c>
       <c r="E3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -5584,18 +5607,18 @@
         <v>842</v>
       </c>
       <c r="C4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D4">
         <v>624</v>
       </c>
       <c r="E4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B5">
         <v>825</v>
@@ -5607,12 +5630,12 @@
         <v>580</v>
       </c>
       <c r="E5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B6">
         <v>638</v>
@@ -5624,7 +5647,7 @@
         <v>432</v>
       </c>
       <c r="E6" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -5641,7 +5664,7 @@
         <v>402</v>
       </c>
       <c r="E7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -5658,7 +5681,7 @@
         <v>402</v>
       </c>
       <c r="E8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -5669,13 +5692,13 @@
         <v>812</v>
       </c>
       <c r="C9" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D9">
         <v>606</v>
       </c>
       <c r="E9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -5692,7 +5715,7 @@
         <v>228</v>
       </c>
       <c r="E10" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -5703,47 +5726,47 @@
         <v>638</v>
       </c>
       <c r="C11" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D11">
         <v>606</v>
       </c>
       <c r="E11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B12">
         <v>866</v>
       </c>
       <c r="C12" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D12">
         <v>621</v>
       </c>
       <c r="E12" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B13">
         <v>896</v>
       </c>
       <c r="C13" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D13">
         <v>651</v>
       </c>
       <c r="E13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -5754,7 +5777,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABF9D4FB-A849-439C-802C-83D42FDCE3EA}">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="30.25" customWidth="1"/>
@@ -5766,7 +5789,7 @@
         <v>111</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C1" s="8" t="s">
         <v>64</v>
@@ -5774,7 +5797,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B2" t="s">
         <v>80</v>
@@ -5782,7 +5805,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B3" t="s">
         <v>84</v>
@@ -5790,7 +5813,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B4" t="s">
         <v>80</v>
@@ -5798,7 +5821,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B5" t="s">
         <v>84</v>
@@ -5806,7 +5829,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B6" t="s">
         <v>44</v>
@@ -5814,7 +5837,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B7" t="s">
         <v>46</v>
@@ -5822,15 +5845,15 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
+        <v>201</v>
+      </c>
+      <c r="B8" t="s">
         <v>202</v>
-      </c>
-      <c r="B8" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B9" t="s">
         <v>47</v>
@@ -5838,15 +5861,15 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B10" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B11" t="s">
         <v>36</v>
@@ -5854,18 +5877,18 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B12" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -5873,7 +5896,7 @@
         <v>112</v>
       </c>
       <c r="B14" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C14" t="s">
         <v>114</v>
@@ -5884,7 +5907,7 @@
         <v>113</v>
       </c>
       <c r="B15" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C15" t="s">
         <v>115</v>
@@ -5892,7 +5915,7 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B16" t="s">
         <v>44</v>
@@ -5900,7 +5923,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B17" t="s">
         <v>46</v>
@@ -5908,15 +5931,15 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B18" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B19" t="s">
         <v>47</v>
@@ -5924,31 +5947,31 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B20" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B21" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B22" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B23" t="s">
         <v>36</v>
@@ -5956,7 +5979,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B24" t="s">
         <v>17</v>
@@ -5964,15 +5987,15 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B25" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B26" t="s">
         <v>36</v>
@@ -5980,15 +6003,15 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B27" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B28" t="s">
         <v>18</v>
@@ -5996,32 +6019,32 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B29" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C29" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B30" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C30" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B31" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -6070,7 +6093,7 @@
         <v>113</v>
       </c>
       <c r="B36" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C36" t="s">
         <v>119</v>
@@ -6086,10 +6109,10 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" s="7" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B38" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C38" t="s">
         <v>110</v>
@@ -6097,18 +6120,50 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" s="7" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B39" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="7" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B40" t="s">
-        <v>249</v>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="B41" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="B42" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="B43" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="B44" t="s">
+        <v>295</v>
       </c>
     </row>
   </sheetData>
@@ -6146,7 +6201,7 @@
         <v>162</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>159</v>
@@ -6157,30 +6212,30 @@
     </row>
     <row r="2" spans="1:6" ht="33">
       <c r="A2" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>163</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>164</v>
       </c>
       <c r="C2" s="5">
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E2" s="5">
         <v>0.2</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="B3" s="7" t="s">
         <v>163</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>164</v>
       </c>
       <c r="C3" s="5">
         <v>0</v>
@@ -6192,15 +6247,15 @@
         <v>0.2</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="49.5">
       <c r="A4" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>163</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>164</v>
       </c>
       <c r="C4" s="5">
         <v>0</v>
@@ -6212,15 +6267,15 @@
         <v>0.25</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="33">
       <c r="A5" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="B5" s="7" t="s">
         <v>163</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>164</v>
       </c>
       <c r="C5" s="5">
         <v>0</v>
@@ -6232,95 +6287,95 @@
         <v>0.25</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="33">
       <c r="A6" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="C6" t="s">
         <v>170</v>
       </c>
-      <c r="C6" t="s">
-        <v>171</v>
-      </c>
       <c r="D6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E6" s="5">
         <v>0.05</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="49.5">
       <c r="A7" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C7" s="5">
         <v>0</v>
       </c>
       <c r="D7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E7" s="5">
         <v>0.2</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="33">
       <c r="A8" s="7" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C8" s="5">
         <v>0</v>
       </c>
       <c r="D8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E8" s="5">
         <v>0.2</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="33">
       <c r="A9" s="7" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C9" s="5">
         <v>0</v>
       </c>
       <c r="D9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E9" s="5">
         <v>0.2</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="49.5">
       <c r="A10" s="7" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C10" s="5">
         <v>0</v>
@@ -6332,15 +6387,15 @@
         <v>0.25</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="33">
       <c r="A11" s="7" t="s">
-        <v>222</v>
+        <v>296</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>225</v>
+        <v>169</v>
       </c>
       <c r="C11" s="5">
         <v>0</v>
@@ -6352,27 +6407,27 @@
         <v>0.25</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="33">
       <c r="A12" s="7" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C12" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D12" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E12" s="5">
         <v>0.05</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -6400,7 +6455,7 @@
         <v>156</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>121</v>
+        <v>297</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>122</v>
@@ -6408,13 +6463,13 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>123</v>
+        <v>193</v>
       </c>
       <c r="D2" s="7" t="b">
         <v>1</v>
@@ -6425,7 +6480,7 @@
         <v>125</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C3" s="7" t="s">
         <v>123</v>
@@ -6436,13 +6491,13 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>193</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>257</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>194</v>
       </c>
       <c r="D4" s="7" t="b">
         <v>1</v>
@@ -6450,13 +6505,13 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D5" s="7" t="b">
         <v>1</v>
@@ -6464,13 +6519,13 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="7" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D6" s="7" t="b">
         <v>1</v>
@@ -6478,13 +6533,13 @@
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="7" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B7" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D7" s="7" t="b">
         <v>1</v>
@@ -6516,7 +6571,7 @@
         <v>121</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>122</v>
+        <v>291</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>159</v>
@@ -6527,13 +6582,13 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>257</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D2" s="7" t="b">
         <v>1</v>
@@ -6544,13 +6599,13 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D3" s="7" t="b">
         <v>1</v>
@@ -6561,13 +6616,13 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B4" t="s">
         <v>82</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D4" t="b">
         <v>0</v>
@@ -6578,13 +6633,13 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="7" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D5" t="b">
         <v>0</v>
@@ -6595,13 +6650,13 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="7" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D6" t="b">
         <v>0</v>
@@ -6612,13 +6667,13 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="7" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B7" t="s">
         <v>93</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D7" t="b">
         <v>0</v>
@@ -6629,13 +6684,13 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="7" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B8" t="s">
         <v>91</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D8" t="b">
         <v>0</v>
@@ -6646,13 +6701,13 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="7" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B9" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D9" t="b">
         <v>0</v>
@@ -6668,23 +6723,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="f82b70a8-9591-478e-a6d5-bf315b83c485" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="ドキュメント" ma:contentTypeID="0x010100B01D25D17823C344A9D69518AF56DC62" ma:contentTypeVersion="6" ma:contentTypeDescription="新しいドキュメントを作成します。" ma:contentTypeScope="" ma:versionID="f29605d1c82d3d43c74cd3efc573dd15">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="f82b70a8-9591-478e-a6d5-bf315b83c485" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d7d0483a01e3419b531383906934819f" ns3:_="">
     <xsd:import namespace="f82b70a8-9591-478e-a6d5-bf315b83c485"/>
@@ -6840,10 +6878,37 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="f82b70a8-9591-478e-a6d5-bf315b83c485" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F80E8E46-C8F1-4EA0-9D75-58D6A3F6209E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3840DE93-E5DB-49F7-A595-E7AEB960EE63}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f82b70a8-9591-478e-a6d5-bf315b83c485"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6865,19 +6930,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3840DE93-E5DB-49F7-A595-E7AEB960EE63}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F80E8E46-C8F1-4EA0-9D75-58D6A3F6209E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f82b70a8-9591-478e-a6d5-bf315b83c485"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>